<commit_message>
Update data sheet and file names for first batch of recordings
</commit_message>
<xml_diff>
--- a/Vocalization_recording_data.xlsx
+++ b/Vocalization_recording_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/omer/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2a96053f85c76562/Documents/GitHub/Vocalizations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DC0BFB-3689-C44E-90C6-979D1331AE58}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{26DC0BFB-3689-C44E-90C6-979D1331AE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7963236C-ED8F-4AFD-BC8D-DB7DE54E9A0E}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17080" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>CAGE NUMBER</t>
   </si>
@@ -54,7 +54,16 @@
     <t>???</t>
   </si>
   <si>
-    <t>T0000009</t>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>marked_853626_260625.wav</t>
+  </si>
+  <si>
+    <t>unmarked_83626_260604.wav</t>
+  </si>
+  <si>
+    <t>unmarked_853626_260625.wav</t>
   </si>
 </sst>
 </file>
@@ -98,9 +107,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -119,9 +131,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -159,7 +171,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -265,7 +277,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -407,7 +419,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -416,9 +428,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90440726-6508-7B45-9053-6C2454E26D68}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="29.08203125" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.1640625" customWidth="1"/>
+    <col min="8" max="8" width="14.08203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -444,29 +463,56 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>853626</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>16</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="E2">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>853626</v>
+      </c>
+      <c r="B3" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="C3" s="2">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>19</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New vocalizations and updating names
Added 6 new vocalizations (4 unscarred, 2 scarred). Corrected filenames.
</commit_message>
<xml_diff>
--- a/Vocalization_recording_data.xlsx
+++ b/Vocalization_recording_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2a96053f85c76562/Documents/GitHub/Vocalizations/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cayma\OneDrive\Documents\GitHub\Vocalizations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{26DC0BFB-3689-C44E-90C6-979D1331AE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7963236C-ED8F-4AFD-BC8D-DB7DE54E9A0E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22C56AFF-B3E7-4B78-9FD8-38F58A352E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>CAGE NUMBER</t>
   </si>
@@ -60,10 +60,28 @@
     <t>marked_853626_260625.wav</t>
   </si>
   <si>
-    <t>unmarked_83626_260604.wav</t>
-  </si>
-  <si>
     <t>unmarked_853626_260625.wav</t>
+  </si>
+  <si>
+    <t>unmarked_857516_260806.wav</t>
+  </si>
+  <si>
+    <t>unmarked_857515_260806.wav</t>
+  </si>
+  <si>
+    <t>marked_857516_260806.wav</t>
+  </si>
+  <si>
+    <t>marked_857515_260806.wav</t>
+  </si>
+  <si>
+    <t>marked_857513_260807.wav</t>
+  </si>
+  <si>
+    <t>unmarked_857513_260807.wav</t>
+  </si>
+  <si>
+    <t>unmarked_853626_260604.wav</t>
   </si>
 </sst>
 </file>
@@ -427,7 +445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90440726-6508-7B45-9053-6C2454E26D68}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="29.08203125" customWidth="1"/>
@@ -500,7 +518,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E3" s="2">
         <v>0</v>
@@ -509,10 +527,128 @@
         <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>857516</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>857516</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>16</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>857515</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>857515</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>857514</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>857514</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>857513</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>16</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>857513</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>16</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding recording and updating records
Another scar group (857514), plus columns for emptyGel and dcnGel groups.
</commit_message>
<xml_diff>
--- a/Vocalization_recording_data.xlsx
+++ b/Vocalization_recording_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2a96053f85c76562/Documents/GitHub/Vocalizations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{22C56AFF-B3E7-4B78-9FD8-38F58A352E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F417048-72CE-480F-BD09-102E0D364DD6}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{22C56AFF-B3E7-4B78-9FD8-38F58A352E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17CCD501-8C47-4553-A71C-B8A76BF4C01D}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>CAGE NUMBER</t>
   </si>
@@ -81,7 +81,40 @@
     <t>unmarked_853626_260604.wav</t>
   </si>
   <si>
-    <t>marked_857514_2608XX.wav</t>
+    <t>unmarked_857516_260827.wav</t>
+  </si>
+  <si>
+    <t>marked_857516_260827.wav</t>
+  </si>
+  <si>
+    <t>marked_857515_260827.wav</t>
+  </si>
+  <si>
+    <t>unmarked_857515_260827.wav</t>
+  </si>
+  <si>
+    <t>marked_857513_260828.wav</t>
+  </si>
+  <si>
+    <t>unmarked_857513_260828.wav</t>
+  </si>
+  <si>
+    <t>marked_857514_260813.wav</t>
+  </si>
+  <si>
+    <t>unmarked_857514_260813.wav</t>
+  </si>
+  <si>
+    <t>marked_857514_260903.wav</t>
+  </si>
+  <si>
+    <t>unmarked_857514_260903.wav</t>
+  </si>
+  <si>
+    <t>EmptyGel</t>
+  </si>
+  <si>
+    <t>DcnGel</t>
   </si>
 </sst>
 </file>
@@ -448,17 +481,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90440726-6508-7B45-9053-6C2454E26D68}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="29.08203125" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.1640625" customWidth="1"/>
-    <col min="8" max="8" width="14.08203125" customWidth="1"/>
+    <col min="5" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="28.1640625" customWidth="1"/>
+    <col min="10" max="10" width="14.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,16 +508,22 @@
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>853626</v>
       </c>
@@ -501,14 +540,20 @@
         <v>1</v>
       </c>
       <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
         <v>19</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>853626</v>
       </c>
@@ -525,14 +570,20 @@
         <v>1</v>
       </c>
       <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
         <v>19</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>857516</v>
       </c>
@@ -548,14 +599,20 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>19</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>857516</v>
       </c>
@@ -571,14 +628,20 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5">
         <v>19</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I5" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>857515</v>
       </c>
@@ -594,14 +657,20 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>19</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>857515</v>
       </c>
@@ -617,14 +686,20 @@
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>19</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I7" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>857514</v>
       </c>
@@ -635,17 +710,25 @@
         <v>17</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8">
         <v>20</v>
       </c>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I8" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>857514</v>
       </c>
@@ -656,16 +739,25 @@
         <v>17</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>857513</v>
       </c>
@@ -681,14 +773,20 @@
       <c r="E10">
         <v>1</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10">
         <v>19</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I10" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>857513</v>
       </c>
@@ -704,11 +802,17 @@
       <c r="E11">
         <v>1</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11">
         <v>19</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>16</v>
+      <c r="I11" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>